<commit_message>
brand-video: Effort Levels tab (levels 1-10, per-film estimates, plan rates as inputs)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ovbscV2XeLVGCnB525Lp4
</commit_message>
<xml_diff>
--- a/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
+++ b/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
@@ -14,6 +14,7 @@
     <sheet name="3 Brand · Master" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Assets" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Style Library" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Effort Levels" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'1 Streamer Stories'!$A$4:$U$13</definedName>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="514">
   <si>
     <t xml:space="preserve">Chobbot media plan · v0.1 (mockup)</t>
   </si>
@@ -1307,16 +1308,303 @@
   </si>
   <si>
     <t xml:space="preserve">Reads as AI-made</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effort levels · what each level costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Levels from the medium-lens-film skill (07_quality_levels.md). Hours are Opus agent-hours of building, estimates until the first film is calibrated. Blue cells are inputs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Looks like</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rendering added at this level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agent-hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final render (GPU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean synced motion graphics, one look</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloom, grain, flash/shake on hits, word-synced type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3–4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minutes (1080p)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simple 3D lit properly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soft shadows, ambient occlusion, real materials, depth of field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4–5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ atmosphere</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fog, god rays, rain on glass, wet reflections, secondary motion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5–6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low–medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Studio ad; mixed style deck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bounce light, PBR bloom, flares, lens dirt; 3–5 switch styles + material transitions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6–7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dressed sets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 fully dressed environments, lit particles, mosaic of styles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7–8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cinematic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volumetric sky/light, 60 fps adaptive motion blur, 1 hero shot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8–10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium–high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feels shot on film</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Film grain, halation, gate weave, grade per shot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10–11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Directed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camera choreography per shot, a material transition on every cut, nested pull-back ending</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11–13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloth, smoke/ink, voxel destruction, crowds of chat bubbles, sound design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13–14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S++</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2430"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">《光先到》 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2430"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ pdoom 4K</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Every shot a hero shot, 4K60 path-traced look</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14–16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very high (20–60+ GPU-h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan rates (% of a weekly allowance per agent-hour, incl. +30% rework; replace with your own after calibration)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max 5×</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max 20×</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: medium-lens-film skill, references/07_quality_levels.md (branch claude/zealous-newton-7zpeja). Estimates, not measurements.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effort by film (first wave)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Film(s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours each</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pro weeks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max 5× weeks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max 20× weeks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Why this level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-01 (first story)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 · B mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Builds the shared style-deck shaders, the pixel/voxel streamer and kinetic type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-02 … ST-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reuses the deck shaders; new story, song timing, style picks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GN-U1A (first A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 · A depth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Builds the majestic sets: system view, constellations, sky</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GN-U2A … U8A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reuses the A sets; new use case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GN-U1B (first B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 · B+ mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Builds the streamer room in pixel/voxel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GN-U2B … U8B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reuses the room and the deck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 · S depth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The hero film: camera choreography, nested pull-back</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 · A+ mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same beats as A, reuses its assets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weeks = weekly allowances used (1.0 = one full week of that plan). Calibrate on ST-01: note the usage bar before and after, then replace the rates above.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="0.00%"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1402,8 +1690,29 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F2430"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF1F2430"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1437,7 +1746,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDCEBFF"/>
-        <bgColor rgb="FFEEEEEE"/>
+        <bgColor rgb="FFE9ECF2"/>
       </patternFill>
     </fill>
     <fill>
@@ -1461,7 +1770,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEEEEEE"/>
-        <bgColor rgb="FFF3F3F3"/>
+        <bgColor rgb="FFE9ECF2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9ECF2"/>
+        <bgColor rgb="FFEEEEEE"/>
       </patternFill>
     </fill>
   </fills>
@@ -1514,7 +1829,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1589,6 +1904,34 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1739,7 +2082,7 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFF3F3F3"/>
+      <rgbColor rgb="FFEEEEEE"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -1747,7 +2090,7 @@
       <rgbColor rgb="FFDCEBFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF0F6FDE"/>
       <rgbColor rgb="FFC9CED8"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -1758,10 +2101,10 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFEEEEEE"/>
+      <rgbColor rgb="FFE9ECF2"/>
       <rgbColor rgb="FFD5F2DC"/>
       <rgbColor rgb="FFFFE7B3"/>
-      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFF3F3F3"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFF8D3D3"/>
@@ -5850,4 +6193,658 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF0F6FDE"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="62"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>475</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="20" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>0.065</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>0.013</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>0.0033</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="16" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>489</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>493</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <f aca="false">D24*E24</f>
+        <v>6.5</v>
+      </c>
+      <c r="G24" s="23" t="n">
+        <f aca="false">F24*$B$17</f>
+        <v>0.4225</v>
+      </c>
+      <c r="H24" s="23" t="n">
+        <f aca="false">F24*$B$18</f>
+        <v>0.0845</v>
+      </c>
+      <c r="I24" s="23" t="n">
+        <f aca="false">F24*$B$19</f>
+        <v>0.02145</v>
+      </c>
+      <c r="J24" s="5" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="E25" s="22" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <f aca="false">D25*E25</f>
+        <v>17.5</v>
+      </c>
+      <c r="G25" s="23" t="n">
+        <f aca="false">F25*$B$17</f>
+        <v>1.1375</v>
+      </c>
+      <c r="H25" s="23" t="n">
+        <f aca="false">F25*$B$18</f>
+        <v>0.2275</v>
+      </c>
+      <c r="I25" s="23" t="n">
+        <f aca="false">F25*$B$19</f>
+        <v>0.05775</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D26" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <f aca="false">D26*E26</f>
+        <v>9</v>
+      </c>
+      <c r="G26" s="23" t="n">
+        <f aca="false">F26*$B$17</f>
+        <v>0.585</v>
+      </c>
+      <c r="H26" s="23" t="n">
+        <f aca="false">F26*$B$18</f>
+        <v>0.117</v>
+      </c>
+      <c r="I26" s="23" t="n">
+        <f aca="false">F26*$B$19</f>
+        <v>0.0297</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D27" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="E27" s="22" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <f aca="false">D27*E27</f>
+        <v>24.5</v>
+      </c>
+      <c r="G27" s="23" t="n">
+        <f aca="false">F27*$B$17</f>
+        <v>1.5925</v>
+      </c>
+      <c r="H27" s="23" t="n">
+        <f aca="false">F27*$B$18</f>
+        <v>0.3185</v>
+      </c>
+      <c r="I27" s="23" t="n">
+        <f aca="false">F27*$B$19</f>
+        <v>0.08085</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="D28" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <f aca="false">D28*E28</f>
+        <v>4</v>
+      </c>
+      <c r="G28" s="23" t="n">
+        <f aca="false">F28*$B$17</f>
+        <v>0.26</v>
+      </c>
+      <c r="H28" s="23" t="n">
+        <f aca="false">F28*$B$18</f>
+        <v>0.052</v>
+      </c>
+      <c r="I28" s="23" t="n">
+        <f aca="false">F28*$B$19</f>
+        <v>0.0132</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="D29" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="E29" s="22" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <f aca="false">D29*E29</f>
+        <v>17.5</v>
+      </c>
+      <c r="G29" s="23" t="n">
+        <f aca="false">F29*$B$17</f>
+        <v>1.1375</v>
+      </c>
+      <c r="H29" s="23" t="n">
+        <f aca="false">F29*$B$18</f>
+        <v>0.2275</v>
+      </c>
+      <c r="I29" s="23" t="n">
+        <f aca="false">F29*$B$19</f>
+        <v>0.05775</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>508</v>
+      </c>
+      <c r="D30" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <f aca="false">D30*E30</f>
+        <v>12</v>
+      </c>
+      <c r="G30" s="23" t="n">
+        <f aca="false">F30*$B$17</f>
+        <v>0.78</v>
+      </c>
+      <c r="H30" s="23" t="n">
+        <f aca="false">F30*$B$18</f>
+        <v>0.156</v>
+      </c>
+      <c r="I30" s="23" t="n">
+        <f aca="false">F30*$B$19</f>
+        <v>0.0396</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>510</v>
+      </c>
+      <c r="D31" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <f aca="false">D31*E31</f>
+        <v>7</v>
+      </c>
+      <c r="G31" s="23" t="n">
+        <f aca="false">F31*$B$17</f>
+        <v>0.455</v>
+      </c>
+      <c r="H31" s="23" t="n">
+        <f aca="false">F31*$B$18</f>
+        <v>0.091</v>
+      </c>
+      <c r="I31" s="23" t="n">
+        <f aca="false">F31*$B$19</f>
+        <v>0.0231</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="24" t="s">
+        <v>512</v>
+      </c>
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24" t="n">
+        <f aca="false">SUM(D24:D31)</f>
+        <v>26</v>
+      </c>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24" t="n">
+        <f aca="false">SUM(F24:F31)</f>
+        <v>98</v>
+      </c>
+      <c r="G32" s="25" t="n">
+        <f aca="false">SUM(G24:G31)</f>
+        <v>6.37</v>
+      </c>
+      <c r="H32" s="25" t="n">
+        <f aca="false">SUM(H24:H31)</f>
+        <v>1.274</v>
+      </c>
+      <c r="I32" s="25" t="n">
+        <f aca="false">SUM(I24:I31)</f>
+        <v>0.3234</v>
+      </c>
+      <c r="J32" s="24"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="16" t="s">
+        <v>513</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
brand-video: ST-01 'The train ride' test script v0.1 (brief, beat sheet, lyrics, song brief)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ovbscV2XeLVGCnB525Lp4
</commit_message>
<xml_diff>
--- a/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
+++ b/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="522">
   <si>
     <t xml:space="preserve">Chobbot media plan · v0.1 (mockup)</t>
   </si>
@@ -308,19 +308,43 @@
     <t xml:space="preserve">ST-01</t>
   </si>
   <si>
-    <t xml:space="preserve">Pixel art → Papercut · Neon line · Constellations · Halftone</t>
+    <t xml:space="preserve">The train ride (TEST film, level 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.reddit.com/r/Twitch/comments/1pujw7y/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A desk-bound game streamer streams IRL at Christmas, peaks at 3 viewers; one viewer watches the train ride until the signal drops, then says it was amazing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8, 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pixel art → Neon line · Halftone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warm lo-fi indie pop, 120 BPM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anonymised retelling; ask the author before publishing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Script: docs/scripts/ST-01_train-ride.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voxel diorama → CRT/VHS · LED dot-matrix · Kinetic type · Stained glass</t>
   </si>
   <si>
     <t xml:space="preserve">30–60 s</t>
   </si>
   <si>
     <t xml:space="preserve">Pick from the Story Fisher shortlist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ST-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Voxel diorama → CRT/VHS · LED dot-matrix · Kinetic type · Stained glass</t>
   </si>
   <si>
     <t xml:space="preserve">ST-03</t>
@@ -1993,6 +2017,14 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFE7B3"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill>
           <bgColor rgb="FFFFFFFF"/>
         </patternFill>
@@ -2045,14 +2077,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF8D3D3"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFE7B3"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2797,29 +2821,45 @@
         <v>89</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
+      <c r="B6" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="H6" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="I6" s="18"/>
+        <v>95</v>
+      </c>
+      <c r="I6" s="18" t="s">
+        <v>96</v>
+      </c>
       <c r="J6" s="5" t="s">
         <v>85</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="L6" s="18"/>
+        <v>97</v>
+      </c>
+      <c r="L6" s="18" t="s">
+        <v>98</v>
+      </c>
       <c r="M6" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>38</v>
@@ -2834,15 +2874,17 @@
         <v>38</v>
       </c>
       <c r="R6" s="18"/>
-      <c r="S6" s="5"/>
+      <c r="S6" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="T6" s="18"/>
       <c r="U6" s="18" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B7" s="18"/>
       <c r="C7" s="18"/>
@@ -2851,14 +2893,14 @@
       <c r="F7" s="18"/>
       <c r="G7" s="18"/>
       <c r="H7" s="5" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="I7" s="18"/>
       <c r="J7" s="5" t="s">
         <v>85</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="L7" s="18"/>
       <c r="M7" s="5" t="s">
@@ -2880,12 +2922,12 @@
       <c r="S7" s="5"/>
       <c r="T7" s="18"/>
       <c r="U7" s="18" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="B8" s="18"/>
       <c r="C8" s="18"/>
@@ -2894,14 +2936,14 @@
       <c r="F8" s="18"/>
       <c r="G8" s="18"/>
       <c r="H8" s="5" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="I8" s="18"/>
       <c r="J8" s="5" t="s">
         <v>85</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="L8" s="18"/>
       <c r="M8" s="5" t="s">
@@ -2923,12 +2965,12 @@
       <c r="S8" s="5"/>
       <c r="T8" s="18"/>
       <c r="U8" s="18" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="B9" s="18"/>
       <c r="C9" s="18"/>
@@ -2937,14 +2979,14 @@
       <c r="F9" s="18"/>
       <c r="G9" s="18"/>
       <c r="H9" s="5" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="I9" s="18"/>
       <c r="J9" s="5" t="s">
         <v>85</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="L9" s="18"/>
       <c r="M9" s="5" t="s">
@@ -2966,12 +3008,12 @@
       <c r="S9" s="5"/>
       <c r="T9" s="18"/>
       <c r="U9" s="18" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B10" s="18"/>
       <c r="C10" s="18"/>
@@ -2980,14 +3022,14 @@
       <c r="F10" s="18"/>
       <c r="G10" s="18"/>
       <c r="H10" s="5" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="I10" s="18"/>
       <c r="J10" s="5" t="s">
         <v>85</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="L10" s="18"/>
       <c r="M10" s="5" t="s">
@@ -3009,12 +3051,12 @@
       <c r="S10" s="5"/>
       <c r="T10" s="18"/>
       <c r="U10" s="18" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="B11" s="18"/>
       <c r="C11" s="18"/>
@@ -3023,14 +3065,14 @@
       <c r="F11" s="18"/>
       <c r="G11" s="18"/>
       <c r="H11" s="5" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="I11" s="18"/>
       <c r="J11" s="5" t="s">
         <v>85</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="L11" s="18"/>
       <c r="M11" s="5" t="s">
@@ -3052,12 +3094,12 @@
       <c r="S11" s="5"/>
       <c r="T11" s="18"/>
       <c r="U11" s="18" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="18"/>
@@ -3066,14 +3108,14 @@
       <c r="F12" s="18"/>
       <c r="G12" s="18"/>
       <c r="H12" s="5" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="I12" s="18"/>
       <c r="J12" s="5" t="s">
         <v>85</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="L12" s="18"/>
       <c r="M12" s="5" t="s">
@@ -3095,12 +3137,12 @@
       <c r="S12" s="5"/>
       <c r="T12" s="18"/>
       <c r="U12" s="18" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="18"/>
@@ -3109,14 +3151,14 @@
       <c r="F13" s="18"/>
       <c r="G13" s="18"/>
       <c r="H13" s="5" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="I13" s="18"/>
       <c r="J13" s="5" t="s">
         <v>85</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="L13" s="18"/>
       <c r="M13" s="5" t="s">
@@ -3138,108 +3180,108 @@
       <c r="S13" s="5"/>
       <c r="T13" s="18"/>
       <c r="U13" s="18" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:U13"/>
   <conditionalFormatting sqref="M5:M13">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>M5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>M5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>M5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>M5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>M5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>M5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:N13">
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>N5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>N5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>N5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>N5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>N5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>N5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O5:O13">
-    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>O5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>O5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>O5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>O5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>O5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>O5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P5:P13">
-    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>P5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>P5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>P5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>P5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>P5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>P5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q5:Q13">
-    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>Q5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>Q5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>Q5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>Q5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="30" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="30" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>Q5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="31" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="31" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>Q5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3307,12 +3349,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3320,37 +3362,37 @@
         <v>55</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>61</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="M4" s="4" t="s">
         <v>64</v>
@@ -3385,44 +3427,44 @@
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>82</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="K5" s="18"/>
       <c r="L5" s="5" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="O5" s="5" t="s">
         <v>38</v>
@@ -3445,44 +3487,44 @@
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>82</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="K6" s="18"/>
       <c r="L6" s="5" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>38</v>
@@ -3505,44 +3547,44 @@
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="J7" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="K7" s="18"/>
       <c r="L7" s="5" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="O7" s="5" t="s">
         <v>38</v>
@@ -3565,44 +3607,44 @@
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="H8" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="J8" s="5" t="s">
         <v>142</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>134</v>
       </c>
       <c r="K8" s="18"/>
       <c r="L8" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="N8" s="5" t="s">
         <v>143</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="N8" s="5" t="s">
-        <v>135</v>
       </c>
       <c r="O8" s="5" t="s">
         <v>38</v>
@@ -3625,44 +3667,44 @@
     </row>
     <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="K9" s="18"/>
       <c r="L9" s="5" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="O9" s="5" t="s">
         <v>38</v>
@@ -3685,44 +3727,44 @@
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="K10" s="18"/>
       <c r="L10" s="5" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="O10" s="5" t="s">
         <v>38</v>
@@ -3745,44 +3787,44 @@
     </row>
     <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="K11" s="18"/>
       <c r="L11" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="O11" s="5" t="s">
         <v>38</v>
@@ -3805,44 +3847,44 @@
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="K12" s="18"/>
       <c r="L12" s="5" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="O12" s="5" t="s">
         <v>38</v>
@@ -3865,44 +3907,44 @@
     </row>
     <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="G13" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="I13" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="H13" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>160</v>
-      </c>
       <c r="J13" s="5" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="K13" s="18"/>
       <c r="L13" s="5" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="O13" s="5" t="s">
         <v>38</v>
@@ -3925,44 +3967,44 @@
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="G14" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="I14" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="H14" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>160</v>
-      </c>
       <c r="J14" s="5" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="K14" s="18"/>
       <c r="L14" s="5" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="O14" s="5" t="s">
         <v>38</v>
@@ -3985,44 +4027,44 @@
     </row>
     <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="K15" s="18"/>
       <c r="L15" s="5" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="O15" s="5" t="s">
         <v>38</v>
@@ -4045,44 +4087,44 @@
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="K16" s="18"/>
       <c r="L16" s="5" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="O16" s="5" t="s">
         <v>38</v>
@@ -4105,44 +4147,44 @@
     </row>
     <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="K17" s="18"/>
       <c r="L17" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="O17" s="5" t="s">
         <v>38</v>
@@ -4165,44 +4207,44 @@
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>182</v>
-      </c>
       <c r="D18" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="K18" s="18"/>
       <c r="L18" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N18" s="5" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="O18" s="5" t="s">
         <v>38</v>
@@ -4225,44 +4267,44 @@
     </row>
     <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="K19" s="18"/>
       <c r="L19" s="5" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="O19" s="5" t="s">
         <v>38</v>
@@ -4285,44 +4327,44 @@
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="K20" s="18"/>
       <c r="L20" s="5" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N20" s="5" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="O20" s="5" t="s">
         <v>38</v>
@@ -4346,102 +4388,102 @@
   </sheetData>
   <autoFilter ref="A4:V20"/>
   <conditionalFormatting sqref="O5:O20">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>O5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>O5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>O5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>O5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>O5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>O5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P5:P20">
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>P5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>P5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>P5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>P5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>P5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>P5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q5:Q20">
-    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>Q5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>Q5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>Q5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>Q5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>Q5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>Q5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R5:R20">
-    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>R5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>R5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>R5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>R5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>R5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>R5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S5:S20">
-    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>S5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>S5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>S5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>S5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="30" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="30" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>S5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="31" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="31" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>S5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4504,12 +4546,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4517,13 +4559,13 @@
         <v>55</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>65</v>
@@ -4532,7 +4574,7 @@
         <v>64</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>67</v>
@@ -4561,25 +4603,25 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>38</v>
@@ -4599,30 +4641,30 @@
       <c r="M5" s="18"/>
       <c r="N5" s="18"/>
       <c r="O5" s="18" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>38</v>
@@ -4642,38 +4684,38 @@
       <c r="M6" s="18"/>
       <c r="N6" s="18"/>
       <c r="O6" s="18" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>75</v>
@@ -4684,22 +4726,22 @@
         <v>1</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>38</v>
@@ -4711,22 +4753,22 @@
         <v>2</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>38</v>
@@ -4738,22 +4780,22 @@
         <v>3</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>38</v>
@@ -4765,22 +4807,22 @@
         <v>4</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>38</v>
@@ -4792,22 +4834,22 @@
         <v>5</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>38</v>
@@ -4817,122 +4859,122 @@
   </sheetData>
   <autoFilter ref="A9:I14"/>
   <conditionalFormatting sqref="H5:H6">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>H5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>H5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>H5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>H5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>H5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>H5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I6">
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>I5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>I5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>I5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>I5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>I5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>I5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:J6">
-    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>J5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>J5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>J5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>J5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>J5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>J5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5:K6">
-    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>K5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>K5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>K5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>K5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>K5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>K5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L5:L6">
-    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>L5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>L5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>L5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>L5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="30" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="30" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>L5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="31" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="31" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>L5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:H14">
-    <cfRule type="expression" priority="32" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="32" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>H10="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="33" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="33" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>H10="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="34" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="34" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>H10="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="35" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="35" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>H10="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="36" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="36" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>H10="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="37" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="37" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>H10="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4995,38 +5037,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>74</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>75</v>
@@ -5034,19 +5076,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>38</v>
@@ -5054,24 +5096,24 @@
       <c r="G5" s="18"/>
       <c r="H5" s="18"/>
       <c r="I5" s="18" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>38</v>
@@ -5082,16 +5124,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
@@ -5103,19 +5145,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>269</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>261</v>
-      </c>
       <c r="C8" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>38</v>
@@ -5123,21 +5165,21 @@
       <c r="G8" s="18"/>
       <c r="H8" s="18"/>
       <c r="I8" s="18" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5" t="s">
@@ -5146,24 +5188,24 @@
       <c r="G9" s="18"/>
       <c r="H9" s="18"/>
       <c r="I9" s="18" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>38</v>
@@ -5171,24 +5213,24 @@
       <c r="G10" s="18"/>
       <c r="H10" s="18"/>
       <c r="I10" s="18" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>38</v>
@@ -5196,24 +5238,24 @@
       <c r="G11" s="18"/>
       <c r="H11" s="18"/>
       <c r="I11" s="18" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>38</v>
@@ -5221,21 +5263,21 @@
       <c r="G12" s="18"/>
       <c r="H12" s="18"/>
       <c r="I12" s="18" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5" t="s">
@@ -5244,21 +5286,21 @@
       <c r="G13" s="18"/>
       <c r="H13" s="18"/>
       <c r="I13" s="18" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5" t="s">
@@ -5267,21 +5309,21 @@
       <c r="G14" s="18"/>
       <c r="H14" s="18"/>
       <c r="I14" s="18" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
@@ -5290,21 +5332,21 @@
       <c r="G15" s="18"/>
       <c r="H15" s="18"/>
       <c r="I15" s="18" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5" t="s">
@@ -5313,21 +5355,21 @@
       <c r="G16" s="18"/>
       <c r="H16" s="18"/>
       <c r="I16" s="18" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="E17" s="5"/>
       <c r="F17" s="5" t="s">
@@ -5336,24 +5378,24 @@
       <c r="G17" s="18"/>
       <c r="H17" s="18"/>
       <c r="I17" s="18" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="F18" s="5" t="s">
         <v>38</v>
@@ -5361,24 +5403,24 @@
       <c r="G18" s="18"/>
       <c r="H18" s="18"/>
       <c r="I18" s="18" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>38</v>
@@ -5386,24 +5428,24 @@
       <c r="G19" s="18"/>
       <c r="H19" s="18"/>
       <c r="I19" s="18" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="F20" s="5" t="s">
         <v>38</v>
@@ -5414,19 +5456,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>39</v>
@@ -5434,24 +5476,24 @@
       <c r="G21" s="18"/>
       <c r="H21" s="18"/>
       <c r="I21" s="18" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>38</v>
@@ -5459,24 +5501,24 @@
       <c r="G22" s="18"/>
       <c r="H22" s="18"/>
       <c r="I22" s="18" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>38</v>
@@ -5484,24 +5526,24 @@
       <c r="G23" s="18"/>
       <c r="H23" s="18"/>
       <c r="I23" s="18" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>38</v>
@@ -5509,21 +5551,21 @@
       <c r="G24" s="18"/>
       <c r="H24" s="18"/>
       <c r="I24" s="18" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="E25" s="5"/>
       <c r="F25" s="5" t="s">
@@ -5532,28 +5574,28 @@
       <c r="G25" s="18"/>
       <c r="H25" s="18"/>
       <c r="I25" s="18" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:I25"/>
   <conditionalFormatting sqref="F5:F25">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>F5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>F5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>F5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>F5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>F5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>F5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5594,32 +5636,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>75</v>
@@ -5627,65 +5669,65 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>38</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>38</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>38</v>
@@ -5694,19 +5736,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>38</v>
@@ -5715,19 +5757,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>38</v>
@@ -5736,19 +5778,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>38</v>
@@ -5757,42 +5799,42 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>38</v>
       </c>
       <c r="G11" s="18" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>38</v>
@@ -5801,19 +5843,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>38</v>
@@ -5822,19 +5864,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>38</v>
@@ -5843,19 +5885,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>38</v>
@@ -5864,19 +5906,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="F16" s="5" t="s">
         <v>38</v>
@@ -5885,19 +5927,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>38</v>
@@ -5906,65 +5948,65 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="F18" s="5" t="s">
         <v>38</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>38</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="F20" s="5" t="s">
         <v>38</v>
@@ -5973,42 +6015,42 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>38</v>
       </c>
       <c r="G21" s="18" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>38</v>
@@ -6017,19 +6059,19 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>38</v>
@@ -6038,19 +6080,19 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>38</v>
@@ -6059,19 +6101,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="D25" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="E25" s="5" t="s">
         <v>415</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>407</v>
       </c>
       <c r="F25" s="5" t="s">
         <v>38</v>
@@ -6080,19 +6122,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>38</v>
@@ -6101,80 +6143,80 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="F27" s="5" t="s">
         <v>43</v>
       </c>
       <c r="G27" s="18" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="F28" s="5" t="s">
         <v>43</v>
       </c>
       <c r="G28" s="18" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:G28"/>
   <conditionalFormatting sqref="F5:F28">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>F5="Not started"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>F5="In progress"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>F5="Review"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>F5="Approved"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>F5="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>F5="N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:B28">
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>B5="A · use freely"</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>B5="B · short holds / backgrounds"</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>B5="C · avoid"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6217,32 +6259,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6250,19 +6292,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6270,19 +6312,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6290,19 +6332,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6310,19 +6352,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6330,19 +6372,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6350,19 +6392,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>458</v>
+        <v>466</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6370,19 +6412,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6390,19 +6432,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>465</v>
+        <v>473</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>467</v>
+        <v>475</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>468</v>
+        <v>476</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6410,19 +6452,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>469</v>
+        <v>477</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>470</v>
+        <v>478</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>471</v>
+        <v>479</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>473</v>
+        <v>481</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6430,29 +6472,29 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>475</v>
+        <v>483</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>476</v>
+        <v>484</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>478</v>
+        <v>486</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>479</v>
+        <v>487</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="B17" s="21" t="n">
         <v>0.065</v>
@@ -6460,7 +6502,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>481</v>
+        <v>489</v>
       </c>
       <c r="B18" s="21" t="n">
         <v>0.013</v>
@@ -6468,7 +6510,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>482</v>
+        <v>490</v>
       </c>
       <c r="B19" s="21" t="n">
         <v>0.0033</v>
@@ -6476,55 +6518,55 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>483</v>
+        <v>491</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>484</v>
+        <v>492</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>485</v>
+        <v>493</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>486</v>
+        <v>494</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>487</v>
+        <v>495</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>488</v>
+        <v>496</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>489</v>
+        <v>497</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>490</v>
+        <v>498</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>491</v>
+        <v>499</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>492</v>
+        <v>500</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>493</v>
+        <v>501</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>494</v>
+        <v>502</v>
       </c>
       <c r="D24" s="22" t="n">
         <v>1</v>
@@ -6549,18 +6591,18 @@
         <v>0.02145</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>496</v>
+        <v>504</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>494</v>
+        <v>502</v>
       </c>
       <c r="D25" s="22" t="n">
         <v>7</v>
@@ -6585,18 +6627,18 @@
         <v>0.05775</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>497</v>
+        <v>505</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>498</v>
+        <v>506</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>499</v>
+        <v>507</v>
       </c>
       <c r="D26" s="22" t="n">
         <v>1</v>
@@ -6621,18 +6663,18 @@
         <v>0.0297</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>500</v>
+        <v>508</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>501</v>
+        <v>509</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>499</v>
+        <v>507</v>
       </c>
       <c r="D27" s="22" t="n">
         <v>7</v>
@@ -6657,18 +6699,18 @@
         <v>0.08085</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>503</v>
+        <v>511</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>504</v>
+        <v>512</v>
       </c>
       <c r="D28" s="22" t="n">
         <v>1</v>
@@ -6693,18 +6735,18 @@
         <v>0.0132</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>505</v>
+        <v>513</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>504</v>
+        <v>512</v>
       </c>
       <c r="D29" s="22" t="n">
         <v>7</v>
@@ -6729,18 +6771,18 @@
         <v>0.05775</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>508</v>
+        <v>516</v>
       </c>
       <c r="D30" s="22" t="n">
         <v>1</v>
@@ -6765,18 +6807,18 @@
         <v>0.0396</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>509</v>
+        <v>517</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>510</v>
+        <v>518</v>
       </c>
       <c r="D31" s="22" t="n">
         <v>1</v>
@@ -6801,12 +6843,12 @@
         <v>0.0231</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>512</v>
+        <v>520</v>
       </c>
       <c r="B32" s="24"/>
       <c r="C32" s="24"/>
@@ -6835,7 +6877,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
-        <v>513</v>
+        <v>521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
brand-video: level 6 is the minimum for every film
ST-01 script v0.2 at level 6 (dressed street and train sets, volumetric
light, physical night sky, refracting rain, lit particles, 60 fps motion
blur, one hero shot). PIPELINE and TIER_LIST record the rule; the Effort
Levels tab raises Stories and Generic B to level 6 (first wave ~118.5 h).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ovbscV2XeLVGCnB525Lp4
</commit_message>
<xml_diff>
--- a/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
+++ b/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="521">
   <si>
     <t xml:space="preserve">Chobbot media plan · v0.1 (mockup)</t>
   </si>
@@ -308,7 +308,7 @@
     <t xml:space="preserve">ST-01</t>
   </si>
   <si>
-    <t xml:space="preserve">The train ride (TEST film, level 3)</t>
+    <t xml:space="preserve">The train ride (first film, level 6)</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.reddit.com/r/Twitch/comments/1pujw7y/</t>
@@ -1337,7 +1337,7 @@
     <t xml:space="preserve">Effort levels · what each level costs</t>
   </si>
   <si>
-    <t xml:space="preserve">Levels from the medium-lens-film skill (07_quality_levels.md). Hours are Opus agent-hours of building, estimates until the first film is calibrated. Blue cells are inputs.</t>
+    <t xml:space="preserve">Owner rule: level 6 is the minimum for every film. Levels from the medium-lens-film skill (07_quality_levels.md); hours are Opus agent-hours, estimates until ST-01 is calibrated. Blue cells are inputs.</t>
   </si>
   <si>
     <t xml:space="preserve">Level</t>
@@ -1559,16 +1559,16 @@
     <t xml:space="preserve">ST-01 (first story)</t>
   </si>
   <si>
-    <t xml:space="preserve">4 · B mixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Builds the shared style-deck shaders, the pixel/voxel streamer and kinetic type</t>
+    <t xml:space="preserve">6 · A mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Builds the deck shaders, pixel/voxel streamer, kinetic type, volumetrics and motion blur</t>
   </si>
   <si>
     <t xml:space="preserve">ST-02 … ST-08</t>
   </si>
   <si>
-    <t xml:space="preserve">Reuses the deck shaders; new story, song timing, style picks</t>
+    <t xml:space="preserve">Reuses the deck shaders; new story, sets, hero shot, song timing</t>
   </si>
   <si>
     <t xml:space="preserve">GN-U1A (first A)</t>
@@ -1589,10 +1589,7 @@
     <t xml:space="preserve">GN-U1B (first B)</t>
   </si>
   <si>
-    <t xml:space="preserve">5 · B+ mixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Builds the streamer room in pixel/voxel</t>
+    <t xml:space="preserve">Builds the streamer room in pixel/voxel at level 6</t>
   </si>
   <si>
     <t xml:space="preserve">GN-U2B … U8B</t>
@@ -6572,23 +6569,23 @@
         <v>1</v>
       </c>
       <c r="E24" s="22" t="n">
-        <v>6.5</v>
+        <v>9</v>
       </c>
       <c r="F24" s="5" t="n">
         <f aca="false">D24*E24</f>
-        <v>6.5</v>
+        <v>9</v>
       </c>
       <c r="G24" s="23" t="n">
         <f aca="false">F24*$B$17</f>
-        <v>0.4225</v>
+        <v>0.585</v>
       </c>
       <c r="H24" s="23" t="n">
         <f aca="false">F24*$B$18</f>
-        <v>0.0845</v>
+        <v>0.117</v>
       </c>
       <c r="I24" s="23" t="n">
         <f aca="false">F24*$B$19</f>
-        <v>0.02145</v>
+        <v>0.0297</v>
       </c>
       <c r="J24" s="5" t="s">
         <v>503</v>
@@ -6608,23 +6605,23 @@
         <v>7</v>
       </c>
       <c r="E25" s="22" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="F25" s="5" t="n">
         <f aca="false">D25*E25</f>
-        <v>17.5</v>
+        <v>24.5</v>
       </c>
       <c r="G25" s="23" t="n">
         <f aca="false">F25*$B$17</f>
-        <v>1.1375</v>
+        <v>1.5925</v>
       </c>
       <c r="H25" s="23" t="n">
         <f aca="false">F25*$B$18</f>
-        <v>0.2275</v>
+        <v>0.3185</v>
       </c>
       <c r="I25" s="23" t="n">
         <f aca="false">F25*$B$19</f>
-        <v>0.05775</v>
+        <v>0.08085</v>
       </c>
       <c r="J25" s="5" t="s">
         <v>505</v>
@@ -6710,68 +6707,68 @@
         <v>16</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="D28" s="22" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="22" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F28" s="5" t="n">
         <f aca="false">D28*E28</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G28" s="23" t="n">
         <f aca="false">F28*$B$17</f>
-        <v>0.26</v>
+        <v>0.52</v>
       </c>
       <c r="H28" s="23" t="n">
         <f aca="false">F28*$B$18</f>
-        <v>0.052</v>
+        <v>0.104</v>
       </c>
       <c r="I28" s="23" t="n">
         <f aca="false">F28*$B$19</f>
-        <v>0.0132</v>
+        <v>0.0264</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>512</v>
+        <v>502</v>
       </c>
       <c r="D29" s="22" t="n">
         <v>7</v>
       </c>
       <c r="E29" s="22" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="F29" s="5" t="n">
         <f aca="false">D29*E29</f>
-        <v>17.5</v>
+        <v>24.5</v>
       </c>
       <c r="G29" s="23" t="n">
         <f aca="false">F29*$B$17</f>
-        <v>1.1375</v>
+        <v>1.5925</v>
       </c>
       <c r="H29" s="23" t="n">
         <f aca="false">F29*$B$18</f>
-        <v>0.2275</v>
+        <v>0.3185</v>
       </c>
       <c r="I29" s="23" t="n">
         <f aca="false">F29*$B$19</f>
-        <v>0.05775</v>
+        <v>0.08085</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6782,7 +6779,7 @@
         <v>20</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D30" s="22" t="n">
         <v>1</v>
@@ -6807,7 +6804,7 @@
         <v>0.0396</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6818,7 +6815,7 @@
         <v>20</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D31" s="22" t="n">
         <v>1</v>
@@ -6843,12 +6840,12 @@
         <v>0.0231</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B32" s="24"/>
       <c r="C32" s="24"/>
@@ -6859,25 +6856,25 @@
       <c r="E32" s="24"/>
       <c r="F32" s="24" t="n">
         <f aca="false">SUM(F24:F31)</f>
-        <v>98</v>
+        <v>118.5</v>
       </c>
       <c r="G32" s="25" t="n">
         <f aca="false">SUM(G24:G31)</f>
-        <v>6.37</v>
+        <v>7.7025</v>
       </c>
       <c r="H32" s="25" t="n">
         <f aca="false">SUM(H24:H31)</f>
-        <v>1.274</v>
+        <v>1.5405</v>
       </c>
       <c r="I32" s="25" t="n">
         <f aca="false">SUM(I24:I31)</f>
-        <v>0.3234</v>
+        <v>0.39105</v>
       </c>
       <c r="J32" s="24"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
brand-video: ST-01 approved; v0.4 fact fixes against the full post, permission DM draft
Lyrics and pictures now use only details from the post (Christmas city
tour, the carousel, the viewer's first train, city to farmland, the other
side of the world, 'thanks for being so chill / amazing stream'); removed
invented rain, phone and night. Plan: ST-01 script Approved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ovbscV2XeLVGCnB525Lp4
</commit_message>
<xml_diff>
--- a/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
+++ b/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
@@ -319,7 +319,7 @@
     <t xml:space="preserve">https://www.reddit.com/r/Twitch/comments/1pujw7y/</t>
   </si>
   <si>
-    <t xml:space="preserve">A desk-bound game streamer streams IRL at Christmas, peaks at 3 viewers; one viewer watches the train ride until the signal drops, then says it was amazing.</t>
+    <t xml:space="preserve">Christmas IRL tour, 3 viewers at peak; one viewer, who had never been on a train, watches the city turn to farmland until the signal drops and calls it an amazing stream.</t>
   </si>
   <si>
     <t xml:space="preserve">8, 15</t>
@@ -334,7 +334,7 @@
     <t xml:space="preserve">52 s</t>
   </si>
   <si>
-    <t xml:space="preserve">Anonymised retelling; ask the author before publishing</t>
+    <t xml:space="preserve">Anonymised retelling; permission DM drafted (in the script)</t>
   </si>
   <si>
     <t xml:space="preserve">Script: docs/scripts/ST-01_train-ride.md</t>
@@ -874,7 +874,7 @@
     <t xml:space="preserve">MV</t>
   </si>
   <si>
-    <t xml:space="preserve">0:00–0:03 “Based on a true story” over a slow push into the pixel city (out on the beat). Then: Pixel city at Christmas: a streamer who usually plays games at a desk steps outside, phone up, LIVE. Viewer counter climbs 1, 2, 3. On the evening train, rain streaks the window and the city slides past (hero shot). The signal bars fall, the picture freezes: signal lost. Black. The chat appears big, typed word by word: 'that was amazing. thank you'. Front-page halftone burst: 3 VIEWERS. ENOUGH. Back on the platform the streamer stops and reads it. The city turns warm; a small spark appears next to the message (companion cameo). End card + credit: Story shared by a streamer on Reddit.</t>
+    <t xml:space="preserve">0:00–0:03 “Based on a true story” over a slow push into the pixel city at dusk (out on the beat). A desk-bound game streamer takes the stream on a Christmas tour of their city: market lights, a castle, a lit carousel. Viewer counter climbs to 3. At the station they are about to end the stream; chat: 'wait, I've never been on a train'. Hero shot: through the window the city falls away into open farmland, fast. The signal bars drop, freeze, black. The chat fills the frame: 'thanks for being so chill. amazing stream'. Halftone burst: 3 VIEWERS. ENOUGH. Pull back over the fields and the globe to one lit window on the other side of the world; a small spark by the message (companion cameo). End card + credit: Story shared by a streamer on Reddit.</t>
   </si>
   <si>
     <t xml:space="preserve">warm lo-fi indie pop, gentle and hopeful, glockenspiel and felt piano, soft synth pads, brushed train-rhythm percussion, soft clear vocal up front, intimate dry production, 120 BPM</t>
@@ -885,27 +885,27 @@
   <si>
     <t xml:space="preserve">[Intro: 2 bars, instrumental, glockenspiel, train rhythm]
 [Verse: soft vocal]
-Took the stream outside on Christmas night
-Phone in my cold hand, city lights
+Took the stream out for Christmas in town
+Market lights, a castle, a carousel
 Three people watching, that's my crowd
 Talking to the street out loud
-Evening train, the windows run
-Rain on the glass, still on, still on
+Train to catch, I'll say goodbye
+"Wait, I've never been on a train"
 [Pre-Chorus: almost spoken]
-Signal fading
+Keep it on till the signal goes
 [Break]
 [Chorus: warm, fuller]
-You stayed till the signal died
-Said it was amazing, on a train at night
-Three is not nothing, three is enough
-Somebody was there, that's what it was
+You watched the city turn to fields
+Your first train, it moved so fast
+Said it was amazing, said thank you
+From the other side of the world
 [Outro: soft]
 That's why I do this
 That's why I do this
 [End]</t>
   </si>
   <si>
-    <t xml:space="preserve">Facts from the post only. Script: docs/scripts/ST-01_train-ride.md</t>
+    <t xml:space="preserve">APPROVED. v0.4: every line checked against the full post. Script: docs/scripts/ST-01_train-ride.md</t>
   </si>
   <si>
     <t xml:space="preserve">The raid from the hero</t>
@@ -2583,7 +2583,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFDCEBFF"/>
+          <fgColor rgb="FFD5F2DC"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2591,7 +2591,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFE7B3"/>
+          <fgColor rgb="FFDCEBFF"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2641,7 +2641,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFD5F2DC"/>
+          <fgColor rgb="FFF8D3D3"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2649,7 +2649,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF8D3D3"/>
+          <fgColor rgb="FFFFE7B3"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">COUNTIF('1 Streamer Stories'!M6:M13,"Approved")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="5" t="n">
         <f aca="false">COUNTIF('1 Streamer Stories'!N6:N13,"Approved")</f>
@@ -3441,7 +3441,7 @@
         <v>99</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
brand-video: Story Context results; ST-01 v0.5 and ST-02 enriched from comments and later posts
ST-01: outro uses the poster's own comment (a visitor in your own town,
feeling like a tourist) and the title's 'worthwhile'; end line 'They kept
streaming IRL.' from later posts. ST-02: 450-viewer raid while chasing a PB
with 4 viewers. STORY_FISHER.md: first Story Context run results.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ovbscV2XeLVGCnB525Lp4
</commit_message>
<xml_diff>
--- a/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
+++ b/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
@@ -874,7 +874,7 @@
     <t xml:space="preserve">MV</t>
   </si>
   <si>
-    <t xml:space="preserve">0:00–0:03 “Based on a true story” over a slow push into the pixel city at dusk (out on the beat). A desk-bound game streamer takes the stream on a Christmas tour of their city: market lights, a castle, a lit carousel. Viewer counter climbs to 3. At the station they are about to end the stream; chat: 'wait, I've never been on a train'. Hero shot: through the window the city falls away into open farmland, fast. The signal bars drop, freeze, black. The chat fills the frame: 'thanks for being so chill. amazing stream'. Halftone burst: 3 VIEWERS. ENOUGH. Pull back over the fields and the globe to one lit window on the other side of the world; a small spark by the message (companion cameo). End card + credit: Story shared by a streamer on Reddit.</t>
+    <t xml:space="preserve">0:00–0:03 “Based on a true story” over a slow push into the pixel city at dusk (out on the beat). A desk-bound game streamer takes the stream on a Christmas tour of their city: market lights, a castle, a lit carousel. Viewer counter climbs to 3. At the station they are about to end the stream; chat: 'wait, I've never been on a train'. Hero shot: through the window the city falls away into open farmland, fast. The signal bars drop, freeze, black. The chat fills the frame: 'thanks for being so chill. amazing stream'. Halftone burst: 3 VIEWERS. ENOUGH. Pull back over the fields and the globe to one lit window on the other side of the world; a small spark by the message (companion cameo). Line: They kept streaming IRL. End card + credit: Story shared by a streamer on Reddit.</t>
   </si>
   <si>
     <t xml:space="preserve">warm lo-fi indie pop, gentle and hopeful, glockenspiel and felt piano, soft synth pads, brushed train-rhythm percussion, soft clear vocal up front, intimate dry production, 120 BPM</t>
@@ -900,18 +900,19 @@
 Said it was amazing, said thank you
 From the other side of the world
 [Outro: soft]
-That's why I do this
-That's why I do this
+Like showing a visitor my town
+I saw it like a tourist too
+That's why it's worth it
 [End]</t>
   </si>
   <si>
-    <t xml:space="preserve">APPROVED. v0.4: every line checked against the full post. Script: docs/scripts/ST-01_train-ride.md</t>
+    <t xml:space="preserve">APPROVED. v0.5 (full picture: comments + later posts checked). v0.4: every line checked against the full post. Script: docs/scripts/ST-01_train-ride.md</t>
   </si>
   <si>
     <t xml:space="preserve">The raid from the hero</t>
   </si>
   <si>
-    <t xml:space="preserve">0:00–0:03 “Based on a true story” over the voxel room in the dark (out on the beat). Then: Voxel diorama: 2020, a YouTube video on an old monitor shows a speedrunner in a cowboy hat (voxel, no face). The viewer makes a Twitch account that night and starts streaming retro games. CRT look: Ninja Gaiden-style pixel action, counter at 4 viewers. LED dot-matrix alert: RAID. It is the same speedrunner. The chat floods (kinetic type), stained-glass burst on the chorus, voxel room fills with lights. End card + credit: Story shared by a streamer on Reddit.</t>
+    <t xml:space="preserve">0:00–0:03 “Based on a true story” over the voxel room in the dark (out on the beat). Then: Voxel diorama: 2020, a YouTube video on an old monitor shows a speedrunner in a cowboy hat (voxel, no face). The viewer makes a Twitch account that night and starts streaming retro games. CRT look: Ninja Gaiden-style pixel action, chasing a personal best, counter at 4 viewers. LED dot-matrix alert: RAID · 450. It is the same speedrunner. The chat floods (kinetic type), stained-glass burst on the chorus, voxel room fills with lights. End card + credit: Story shared by a streamer on Reddit.</t>
   </si>
   <si>
     <t xml:space="preserve">chiptune pop-punk, triumphant and fast, 8-bit synth leads with live drums and driving bass, bright clear vocal, punchy modern production, 140 BPM</t>
@@ -924,19 +925,19 @@
 Made an account that very night
 Started streaming the old games
 [Pre-Chorus: building]
-Four people watching, Ninja Gaiden on
+Four people watching, chasing my best
 [Break]
 [Chorus: full band, shout-along]
 Then the raid came in, it was him
+Four hundred fifty people in
 The one who started all of this
-Look who's in my chat tonight
 Look who's watching now
 [Outro]
 Look who's watching now
 [End]</t>
   </si>
   <si>
-    <t xml:space="preserve">Facts from the post (Story Fisher, quality 9). Never name the speedrunner. Check the full post before scripting.</t>
+    <t xml:space="preserve">Full picture checked (75 comments): arc complete, no follow-ups; raid was 450 viewers while chasing a PB with 4. Never name the speedrunner. Not yet approved.</t>
   </si>
   <si>
     <t xml:space="preserve">(pick from the Story Fisher shortlist)</t>
@@ -5682,7 +5683,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="337.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="351" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>91</v>
       </c>

</xml_diff>

<commit_message>
brand-video: ST-01 v0.6 catchier song (hook from second 0, repeated story line), catchiness rules in Suno guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ovbscV2XeLVGCnB525Lp4
</commit_message>
<xml_diff>
--- a/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
+++ b/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
@@ -877,13 +877,13 @@
     <t xml:space="preserve">0:00–0:03 “Based on a true story” over a slow push into the pixel city at dusk (out on the beat). A desk-bound game streamer takes the stream on a Christmas tour of their city: market lights, a castle, a lit carousel. Viewer counter climbs to 3. At the station they are about to end the stream; chat: 'wait, I've never been on a train'. Hero shot: through the window the city falls away into open farmland, fast. The signal bars drop, freeze, black. The chat fills the frame: 'thanks for being so chill. amazing stream'. Halftone burst: 3 VIEWERS. ENOUGH. Pull back over the fields and the globe to one lit window on the other side of the world; a small spark by the message (companion cameo). Line: They kept streaming IRL. End card + credit: Story shared by a streamer on Reddit.</t>
   </si>
   <si>
-    <t xml:space="preserve">warm lo-fi indie pop, gentle and hopeful, glockenspiel and felt piano, soft synth pads, brushed train-rhythm percussion, soft clear vocal up front, intimate dry production, 120 BPM</t>
+    <t xml:space="preserve">catchy upbeat indie pop, warm and hopeful, glockenspiel hook from the first second, train-rhythm drums with handclaps, bright felt piano, clear warm vocal up front, singalong chorus, crisp modern production, 120 BPM</t>
   </si>
   <si>
     <t xml:space="preserve">heavy reverb, autotune, rap verses, spoken word intro, long instrumental intro</t>
   </si>
   <si>
-    <t xml:space="preserve">[Intro: 2 bars, instrumental, glockenspiel, train rhythm]
+    <t xml:space="preserve">[Intro: 2 bars, glockenspiel hook, train-rhythm drums]
 [Verse: soft vocal]
 Took the stream out for Christmas in town
 Market lights, a castle, a carousel
@@ -891,22 +891,23 @@
 Talking to the street out loud
 Train to catch, I'll say goodbye
 "Wait, I've never been on a train"
-[Pre-Chorus: almost spoken]
-Keep it on till the signal goes
+[Pre-Chorus: rising]
+"Can you keep it on?"
 [Break]
-[Chorus: warm, fuller]
+[Chorus: catchy singalong, full drums, glockenspiel hook]
+Keep it on, keep it on, till the signal's gone
 You watched the city turn to fields
 Your first train, it moved so fast
-Said it was amazing, said thank you
-From the other side of the world
-[Outro: soft]
+Keep it on, keep it on, till the signal's gone
+Said it was amazing, from the other side of the world
+[Outro: soft, glockenspiel hook returns]
 Like showing a visitor my town
 I saw it like a tourist too
 That's why it's worth it
 [End]</t>
   </si>
   <si>
-    <t xml:space="preserve">APPROVED. v0.5 (full picture: comments + later posts checked). v0.4: every line checked against the full post. Script: docs/scripts/ST-01_train-ride.md</t>
+    <t xml:space="preserve">APPROVED. v0.6 catchier (hook from second 0, repeated chorus line from the story). v0.5 (full picture: comments + later posts checked). v0.4: every line checked against the full post. Script: docs/scripts/ST-01_train-ride.md</t>
   </si>
   <si>
     <t xml:space="preserve">The raid from the hero</t>
@@ -5683,7 +5684,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="351" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="363.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>91</v>
       </c>

</xml_diff>

<commit_message>
brand-video: beat-timed material transitions, ST-01 timeline with centred cuts, quality band 6-10, style frames approved
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ovbscV2XeLVGCnB525Lp4
</commit_message>
<xml_diff>
--- a/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
+++ b/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
@@ -337,7 +337,7 @@
     <t xml:space="preserve">Anonymised retelling; permission DM drafted (in the script)</t>
   </si>
   <si>
-    <t xml:space="preserve">Script: docs/scripts/ST-01_train-ride.md · 2026-10-04: song approved (master song_with_intro.wav); script v0.7 retimed. Next: style frames.</t>
+    <t xml:space="preserve">Script: docs/scripts/ST-01_train-ride.md · 2026-10-04: song approved (master song_with_intro.wav); script v0.7 retimed. Next: style frames. · 2026-10-04: style frames approved (13 scenes, no on-screen people, the phone is the protagonist); quality band 6–10. Animatic rendering.</t>
   </si>
   <si>
     <t xml:space="preserve">ST-02</t>
@@ -3439,10 +3439,10 @@
         <v>41</v>
       </c>
       <c r="O6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="P6" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="P6" s="6" t="s">
-        <v>38</v>
       </c>
       <c r="Q6" s="6" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
brand-video: step 9 post description with story summary; ST-01 description draft; remove invented 'reconnected' line
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ovbscV2XeLVGCnB525Lp4
</commit_message>
<xml_diff>
--- a/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
+++ b/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1278" uniqueCount="619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="621">
   <si>
     <t xml:space="preserve">Chobbot media plan · v0.1 (mockup)</t>
   </si>
@@ -268,6 +268,9 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
+    <t xml:space="preserve">Post description (short caption)</t>
+  </si>
+  <si>
     <t xml:space="preserve">ST-EX</t>
   </si>
   <si>
@@ -338,6 +341,9 @@
   </si>
   <si>
     <t xml:space="preserve">Script: docs/scripts/ST-01_train-ride.md · 2026-10-04: song approved (master song_with_intro.wav); script v0.7 retimed. Next: style frames. · 2026-10-04: style frames approved (13 scenes, no on-screen people, the phone is the protagonist); quality band 6–10. Animatic rendering.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A streamer's first real IRL. 3 viewers. One of them had never been on a train. Based on a true story.</t>
   </si>
   <si>
     <t xml:space="preserve">ST-02</t>
@@ -3237,7 +3243,7 @@
     <tabColor rgb="FF7A5AF8"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -3257,6 +3263,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3333,43 +3340,46 @@
       <c r="U4" s="5" t="s">
         <v>76</v>
       </c>
+      <c r="V4" s="5" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I5" s="18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J5" s="18" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K5" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="M5" s="18" t="s">
         <v>39</v>
@@ -3388,49 +3398,49 @@
       </c>
       <c r="R5" s="18"/>
       <c r="S5" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="T5" s="18"/>
       <c r="U5" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L6" s="19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M6" s="6" t="s">
         <v>41</v>
@@ -3449,49 +3459,52 @@
       </c>
       <c r="R6" s="19"/>
       <c r="S6" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="T6" s="19"/>
       <c r="U6" s="19" t="s">
-        <v>100</v>
+        <v>101</v>
+      </c>
+      <c r="V6" s="6" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M7" s="6" t="s">
         <v>38</v>
@@ -3510,16 +3523,16 @@
       </c>
       <c r="R7" s="19"/>
       <c r="S7" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="T7" s="19"/>
       <c r="U7" s="19" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="19"/>
@@ -3528,14 +3541,14 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I8" s="19"/>
       <c r="J8" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L8" s="19"/>
       <c r="M8" s="6" t="s">
@@ -3557,12 +3570,12 @@
       <c r="S8" s="6"/>
       <c r="T8" s="19"/>
       <c r="U8" s="19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B9" s="19"/>
       <c r="C9" s="19"/>
@@ -3571,14 +3584,14 @@
       <c r="F9" s="19"/>
       <c r="G9" s="19"/>
       <c r="H9" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I9" s="19"/>
       <c r="J9" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L9" s="19"/>
       <c r="M9" s="6" t="s">
@@ -3600,12 +3613,12 @@
       <c r="S9" s="6"/>
       <c r="T9" s="19"/>
       <c r="U9" s="19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B10" s="19"/>
       <c r="C10" s="19"/>
@@ -3614,14 +3627,14 @@
       <c r="F10" s="19"/>
       <c r="G10" s="19"/>
       <c r="H10" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I10" s="19"/>
       <c r="J10" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L10" s="19"/>
       <c r="M10" s="6" t="s">
@@ -3643,12 +3656,12 @@
       <c r="S10" s="6"/>
       <c r="T10" s="19"/>
       <c r="U10" s="19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B11" s="19"/>
       <c r="C11" s="19"/>
@@ -3657,14 +3670,14 @@
       <c r="F11" s="19"/>
       <c r="G11" s="19"/>
       <c r="H11" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I11" s="19"/>
       <c r="J11" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L11" s="19"/>
       <c r="M11" s="6" t="s">
@@ -3686,12 +3699,12 @@
       <c r="S11" s="6"/>
       <c r="T11" s="19"/>
       <c r="U11" s="19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B12" s="19"/>
       <c r="C12" s="19"/>
@@ -3700,14 +3713,14 @@
       <c r="F12" s="19"/>
       <c r="G12" s="19"/>
       <c r="H12" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I12" s="19"/>
       <c r="J12" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L12" s="19"/>
       <c r="M12" s="6" t="s">
@@ -3729,12 +3742,12 @@
       <c r="S12" s="6"/>
       <c r="T12" s="19"/>
       <c r="U12" s="19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B13" s="19"/>
       <c r="C13" s="19"/>
@@ -3743,14 +3756,14 @@
       <c r="F13" s="19"/>
       <c r="G13" s="19"/>
       <c r="H13" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I13" s="19"/>
       <c r="J13" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="L13" s="19"/>
       <c r="M13" s="6" t="s">
@@ -3772,7 +3785,7 @@
       <c r="S13" s="6"/>
       <c r="T13" s="19"/>
       <c r="U13" s="19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -3941,12 +3954,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3954,37 +3967,37 @@
         <v>56</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>62</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="M4" s="5" t="s">
         <v>65</v>
@@ -4019,44 +4032,44 @@
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K5" s="19"/>
       <c r="L5" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O5" s="6" t="s">
         <v>38</v>
@@ -4079,44 +4092,44 @@
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K6" s="19"/>
       <c r="L6" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O6" s="6" t="s">
         <v>38</v>
@@ -4139,44 +4152,44 @@
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K7" s="19"/>
       <c r="L7" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O7" s="6" t="s">
         <v>38</v>
@@ -4199,44 +4212,44 @@
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="I8" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="J8" s="6" t="s">
         <v>153</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="K8" s="19"/>
       <c r="L8" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O8" s="6" t="s">
         <v>38</v>
@@ -4259,44 +4272,44 @@
     </row>
     <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K9" s="19"/>
       <c r="L9" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O9" s="6" t="s">
         <v>38</v>
@@ -4319,44 +4332,44 @@
     </row>
     <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>167</v>
-      </c>
       <c r="I10" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K10" s="19"/>
       <c r="L10" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O10" s="6" t="s">
         <v>38</v>
@@ -4379,44 +4392,44 @@
     </row>
     <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K11" s="19"/>
       <c r="L11" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O11" s="6" t="s">
         <v>38</v>
@@ -4439,44 +4452,44 @@
     </row>
     <row r="12" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="I12" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>176</v>
-      </c>
       <c r="J12" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K12" s="19"/>
       <c r="L12" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O12" s="6" t="s">
         <v>38</v>
@@ -4499,44 +4512,44 @@
     </row>
     <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K13" s="19"/>
       <c r="L13" s="6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O13" s="6" t="s">
         <v>38</v>
@@ -4559,44 +4572,44 @@
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="H14" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>185</v>
-      </c>
       <c r="I14" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K14" s="19"/>
       <c r="L14" s="6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="M14" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>38</v>
@@ -4619,44 +4632,44 @@
     </row>
     <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K15" s="19"/>
       <c r="L15" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O15" s="6" t="s">
         <v>38</v>
@@ -4679,44 +4692,44 @@
     </row>
     <row r="16" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>194</v>
-      </c>
       <c r="I16" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K16" s="19"/>
       <c r="L16" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>38</v>
@@ -4739,44 +4752,44 @@
     </row>
     <row r="17" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K17" s="19"/>
       <c r="L17" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N17" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O17" s="6" t="s">
         <v>38</v>
@@ -4799,44 +4812,44 @@
     </row>
     <row r="18" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="I18" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>204</v>
-      </c>
       <c r="J18" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K18" s="19"/>
       <c r="L18" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O18" s="6" t="s">
         <v>38</v>
@@ -4859,44 +4872,44 @@
     </row>
     <row r="19" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K19" s="19"/>
       <c r="L19" s="6" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O19" s="6" t="s">
         <v>38</v>
@@ -4919,44 +4932,44 @@
     </row>
     <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>213</v>
-      </c>
       <c r="I20" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="K20" s="19"/>
       <c r="L20" s="6" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O20" s="6" t="s">
         <v>38</v>
@@ -5138,12 +5151,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5151,13 +5164,13 @@
         <v>56</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>66</v>
@@ -5166,7 +5179,7 @@
         <v>65</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>68</v>
@@ -5195,25 +5208,25 @@
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>38</v>
@@ -5233,30 +5246,30 @@
       <c r="M5" s="19"/>
       <c r="N5" s="19"/>
       <c r="O5" s="19" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>38</v>
@@ -5276,38 +5289,38 @@
       <c r="M6" s="19"/>
       <c r="N6" s="19"/>
       <c r="O6" s="19" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>76</v>
@@ -5318,22 +5331,22 @@
         <v>1</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>38</v>
@@ -5345,22 +5358,22 @@
         <v>2</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>38</v>
@@ -5372,22 +5385,22 @@
         <v>3</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>38</v>
@@ -5399,22 +5412,22 @@
         <v>4</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>38</v>
@@ -5426,22 +5439,22 @@
         <v>5</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>38</v>
@@ -5631,12 +5644,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5644,31 +5657,31 @@
         <v>56</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>66</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>76</v>
@@ -5676,856 +5689,856 @@
     </row>
     <row r="5" customFormat="false" ht="363.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>123</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>41</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="298.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>140</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="J6" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="19" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="G7" s="6"/>
       <c r="H7" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>116</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>114</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" s="6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E11" s="6"/>
       <c r="F11" s="6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K11" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K12" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="168.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E13" s="6"/>
       <c r="F13" s="6" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K13" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="298.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="J14" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K14" s="19" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="156" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E15" s="6"/>
       <c r="F15" s="6" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="J15" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K15" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="298.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E16" s="6"/>
       <c r="F16" s="6" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K16" s="19" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="156" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E17" s="6"/>
       <c r="F17" s="6" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K17" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="298.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E18" s="6"/>
       <c r="F18" s="6" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J18" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K18" s="19" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="156" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E19" s="6"/>
       <c r="F19" s="6" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K19" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="298.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="6" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K20" s="19" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="156" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="6" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="J21" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K21" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="298.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="6" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="J22" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="19" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="156" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E23" s="6"/>
       <c r="F23" s="6" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="J23" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K23" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="298.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E24" s="6"/>
       <c r="F24" s="6" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="J24" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K24" s="19" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="156" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E25" s="6"/>
       <c r="F25" s="6" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K25" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="298.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E26" s="6"/>
       <c r="F26" s="6" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="J26" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K26" s="19" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="156" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E27" s="6"/>
       <c r="F27" s="6" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K27" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="298.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E28" s="6"/>
       <c r="F28" s="6" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="J28" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K28" s="19" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="195" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="E29" s="6" t="n">
         <v>90</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="J29" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K29" s="19" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="408.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="E30" s="6" t="n">
         <v>118</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="J30" s="6" t="s">
         <v>38</v>
       </c>
       <c r="K30" s="19" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
   </sheetData>
@@ -6589,38 +6602,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>75</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>76</v>
@@ -6628,19 +6641,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>38</v>
@@ -6648,24 +6661,24 @@
       <c r="G5" s="19"/>
       <c r="H5" s="19"/>
       <c r="I5" s="19" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>371</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>367</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>372</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>369</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>38</v>
@@ -6676,16 +6689,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="6" t="s">
@@ -6697,19 +6710,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>38</v>
@@ -6717,21 +6730,21 @@
       <c r="G8" s="19"/>
       <c r="H8" s="19"/>
       <c r="I8" s="19" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" s="6" t="s">
@@ -6740,24 +6753,24 @@
       <c r="G9" s="19"/>
       <c r="H9" s="19"/>
       <c r="I9" s="19" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>38</v>
@@ -6765,24 +6778,24 @@
       <c r="G10" s="19"/>
       <c r="H10" s="19"/>
       <c r="I10" s="19" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>38</v>
@@ -6790,24 +6803,24 @@
       <c r="G11" s="19"/>
       <c r="H11" s="19"/>
       <c r="I11" s="19" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>389</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>383</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>387</v>
-      </c>
       <c r="D12" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>38</v>
@@ -6815,21 +6828,21 @@
       <c r="G12" s="19"/>
       <c r="H12" s="19"/>
       <c r="I12" s="19" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E13" s="6"/>
       <c r="F13" s="6" t="s">
@@ -6838,21 +6851,21 @@
       <c r="G13" s="19"/>
       <c r="H13" s="19"/>
       <c r="I13" s="19" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6" t="s">
@@ -6861,21 +6874,21 @@
       <c r="G14" s="19"/>
       <c r="H14" s="19"/>
       <c r="I14" s="19" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="E15" s="6"/>
       <c r="F15" s="6" t="s">
@@ -6884,21 +6897,21 @@
       <c r="G15" s="19"/>
       <c r="H15" s="19"/>
       <c r="I15" s="19" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E16" s="6"/>
       <c r="F16" s="6" t="s">
@@ -6907,21 +6920,21 @@
       <c r="G16" s="19"/>
       <c r="H16" s="19"/>
       <c r="I16" s="19" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E17" s="6"/>
       <c r="F17" s="6" t="s">
@@ -6930,24 +6943,24 @@
       <c r="G17" s="19"/>
       <c r="H17" s="19"/>
       <c r="I17" s="19" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>405</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>409</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>403</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>407</v>
-      </c>
       <c r="D18" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>38</v>
@@ -6955,24 +6968,24 @@
       <c r="G18" s="19"/>
       <c r="H18" s="19"/>
       <c r="I18" s="19" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>38</v>
@@ -6980,24 +6993,24 @@
       <c r="G19" s="19"/>
       <c r="H19" s="19"/>
       <c r="I19" s="19" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>413</v>
-      </c>
       <c r="C20" s="6" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>38</v>
@@ -7008,19 +7021,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="F21" s="6" t="s">
         <v>39</v>
@@ -7028,24 +7041,24 @@
       <c r="G21" s="19"/>
       <c r="H21" s="19"/>
       <c r="I21" s="19" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>38</v>
@@ -7053,24 +7066,24 @@
       <c r="G22" s="19"/>
       <c r="H22" s="19"/>
       <c r="I22" s="19" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>428</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>407</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>425</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>426</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>38</v>
@@ -7078,24 +7091,24 @@
       <c r="G23" s="19"/>
       <c r="H23" s="19"/>
       <c r="I23" s="19" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>38</v>
@@ -7103,21 +7116,21 @@
       <c r="G24" s="19"/>
       <c r="H24" s="19"/>
       <c r="I24" s="19" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E25" s="6"/>
       <c r="F25" s="6" t="s">
@@ -7126,7 +7139,7 @@
       <c r="G25" s="19"/>
       <c r="H25" s="19"/>
       <c r="I25" s="19" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
   </sheetData>
@@ -7188,32 +7201,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>76</v>
@@ -7221,65 +7234,65 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>38</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>455</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>447</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>453</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>454</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>450</v>
-      </c>
       <c r="F6" s="6" t="s">
         <v>38</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>38</v>
@@ -7288,19 +7301,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>38</v>
@@ -7309,19 +7322,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>38</v>
@@ -7330,19 +7343,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>38</v>
@@ -7351,42 +7364,42 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>473</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>474</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>471</v>
-      </c>
       <c r="F11" s="6" t="s">
         <v>38</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>38</v>
@@ -7395,19 +7408,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>38</v>
@@ -7416,19 +7429,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>38</v>
@@ -7437,19 +7450,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>447</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>484</v>
-      </c>
       <c r="E15" s="6" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>38</v>
@@ -7458,19 +7471,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>38</v>
@@ -7479,19 +7492,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>38</v>
@@ -7500,65 +7513,65 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>38</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>38</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>38</v>
@@ -7567,42 +7580,42 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="F21" s="6" t="s">
         <v>38</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>38</v>
@@ -7611,19 +7624,19 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>514</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>510</v>
-      </c>
-      <c r="C23" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>515</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>512</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>513</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>38</v>
@@ -7632,19 +7645,19 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>38</v>
@@ -7653,19 +7666,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="F25" s="6" t="s">
         <v>38</v>
@@ -7674,19 +7687,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>38</v>
@@ -7695,48 +7708,48 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>43</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="B28" s="6" t="s">
-        <v>526</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>527</v>
-      </c>
       <c r="D28" s="6" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>43</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
   </sheetData>
@@ -7811,32 +7824,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7844,19 +7857,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7864,19 +7877,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7884,19 +7897,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7904,19 +7917,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7924,19 +7937,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="C9" s="6" t="s">
+        <v>561</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="F9" s="6" t="s">
         <v>559</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>560</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>561</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>557</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7944,19 +7957,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7964,19 +7977,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7984,19 +7997,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>574</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>572</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>573</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>574</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>570</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8004,19 +8017,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8024,29 +8037,29 @@
         <v>10</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B17" s="22" t="n">
         <v>0.065</v>
@@ -8054,7 +8067,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="B18" s="22" t="n">
         <v>0.013</v>
@@ -8062,7 +8075,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="B19" s="22" t="n">
         <v>0.0033</v>
@@ -8070,55 +8083,55 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D24" s="23" t="n">
         <v>1</v>
@@ -8143,18 +8156,18 @@
         <v>0.0297</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D25" s="23" t="n">
         <v>7</v>
@@ -8179,18 +8192,18 @@
         <v>0.08085</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="D26" s="23" t="n">
         <v>1</v>
@@ -8215,18 +8228,18 @@
         <v>0.0297</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="D27" s="23" t="n">
         <v>7</v>
@@ -8251,18 +8264,18 @@
         <v>0.08085</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D28" s="23" t="n">
         <v>1</v>
@@ -8287,18 +8300,18 @@
         <v>0.0264</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D29" s="23" t="n">
         <v>7</v>
@@ -8323,18 +8336,18 @@
         <v>0.08085</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D30" s="23" t="n">
         <v>1</v>
@@ -8359,18 +8372,18 @@
         <v>0.0396</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="D31" s="23" t="n">
         <v>1</v>
@@ -8395,12 +8408,12 @@
         <v>0.0231</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="25" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="B32" s="25"/>
       <c r="C32" s="25"/>
@@ -8429,7 +8442,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ST-01: animatic v4 approved (step 7); media plan updated, build in progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ovbscV2XeLVGCnB525Lp4
</commit_message>
<xml_diff>
--- a/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
+++ b/brand-video/plan/Chobbot_Media_Plan_v0.1.xlsx
@@ -3689,10 +3689,10 @@
         <v>41</v>
       </c>
       <c r="P6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q6" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="Q6" s="6" t="s">
-        <v>38</v>
       </c>
       <c r="R6" s="19"/>
       <c r="S6" s="6" t="s">

</xml_diff>